<commit_message>
adding the new variables to spreadsheet
</commit_message>
<xml_diff>
--- a/backend/variables/variables.xlsx
+++ b/backend/variables/variables.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\falnahas\UNC Charlotte Dropbox\Fatimah Alnahash\ui_git\ui-map-app\backend\variables\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C72FCF6-1576-4004-82E0-9EEFDE77D1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="183">
   <si>
     <t>name</t>
   </si>
@@ -527,14 +533,49 @@
   </si>
   <si>
     <t>Transit Ridership</t>
+  </si>
+  <si>
+    <t>Percent of Population Below Poverty Line</t>
+  </si>
+  <si>
+    <t>Percent of Population Without Health Insurance</t>
+  </si>
+  <si>
+    <t>PercentNotInsuredA</t>
+  </si>
+  <si>
+    <t>PercentMortgageBurdentHouseholdsA</t>
+  </si>
+  <si>
+    <t>Percent of Households Burden with Mortgage Costs</t>
+  </si>
+  <si>
+    <t>Percent of Households Burden with Rent Costs</t>
+  </si>
+  <si>
+    <t>PercentRentCostBurdentHouseholdsA</t>
+  </si>
+  <si>
+    <t>PercentPoverty</t>
+  </si>
+  <si>
+    <t>z_PercentNotInsuredA</t>
+  </si>
+  <si>
+    <t>z_PercentMortgageBurdentHouseholdsA</t>
+  </si>
+  <si>
+    <t>z_PercentRentCostBurdentHouseholdsA</t>
+  </si>
+  <si>
+    <t>z_PercentPoverty</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -552,6 +593,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -583,31 +630,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -618,10 +666,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -659,71 +707,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -751,7 +799,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -774,11 +822,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -787,13 +835,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -803,7 +851,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -812,7 +860,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -821,7 +869,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -829,10 +877,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -897,24 +945,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H95"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="4" width="50.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="8.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="50.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="35" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -940,7 +986,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -959,12 +1005,11 @@
       <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2"/>
       <c r="H2" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -983,12 +1028,11 @@
       <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="2"/>
       <c r="H3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -1007,12 +1051,11 @@
       <c r="F4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="2"/>
       <c r="H4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -1023,28 +1066,22 @@
         <v>23</v>
       </c>
       <c r="F5" s="1"/>
-      <c r="G5" s="2"/>
       <c r="H5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
       <c r="E6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
       <c r="H6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1063,12 +1100,11 @@
       <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="2"/>
       <c r="H7" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -1087,12 +1123,11 @@
       <c r="F8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="2"/>
       <c r="H8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>34</v>
       </c>
@@ -1111,12 +1146,11 @@
       <c r="F9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="2"/>
       <c r="H9" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
@@ -1135,12 +1169,11 @@
       <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="2"/>
       <c r="H10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1159,12 +1192,11 @@
       <c r="F11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="2"/>
       <c r="H11" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
@@ -1183,12 +1215,11 @@
       <c r="F12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="2"/>
       <c r="H12" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -1199,28 +1230,22 @@
         <v>12</v>
       </c>
       <c r="F13" s="1"/>
-      <c r="G13" s="2"/>
       <c r="H13" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H14" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
@@ -1231,12 +1256,11 @@
         <v>23</v>
       </c>
       <c r="F15" s="1"/>
-      <c r="G15" s="2"/>
       <c r="H15" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -1247,12 +1271,11 @@
         <v>23</v>
       </c>
       <c r="F16" s="1"/>
-      <c r="G16" s="2"/>
       <c r="H16" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>55</v>
       </c>
@@ -1271,12 +1294,11 @@
       <c r="F17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="2"/>
       <c r="H17" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>59</v>
       </c>
@@ -1295,12 +1317,11 @@
       <c r="F18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="2"/>
       <c r="H18" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>63</v>
       </c>
@@ -1311,12 +1332,11 @@
         <v>12</v>
       </c>
       <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
       <c r="H19" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>64</v>
       </c>
@@ -1335,12 +1355,11 @@
       <c r="F20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="2"/>
       <c r="H20" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>69</v>
       </c>
@@ -1351,12 +1370,11 @@
         <v>23</v>
       </c>
       <c r="F21" s="1"/>
-      <c r="G21" s="2"/>
       <c r="H21" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>70</v>
       </c>
@@ -1367,12 +1385,11 @@
         <v>12</v>
       </c>
       <c r="F22" s="1"/>
-      <c r="G22" s="2"/>
       <c r="H22" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>71</v>
       </c>
@@ -1391,12 +1408,11 @@
       <c r="F23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="2"/>
       <c r="H23" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>76</v>
       </c>
@@ -1415,12 +1431,11 @@
       <c r="F24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="2"/>
       <c r="H24" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>80</v>
       </c>
@@ -1439,12 +1454,11 @@
       <c r="F25" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="2"/>
       <c r="H25" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>84</v>
       </c>
@@ -1455,12 +1469,11 @@
         <v>12</v>
       </c>
       <c r="F26" s="1"/>
-      <c r="G26" s="2"/>
       <c r="H26" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>85</v>
       </c>
@@ -1471,12 +1484,11 @@
         <v>12</v>
       </c>
       <c r="F27" s="1"/>
-      <c r="G27" s="2"/>
       <c r="H27" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>86</v>
       </c>
@@ -1487,12 +1499,11 @@
         <v>12</v>
       </c>
       <c r="F28" s="1"/>
-      <c r="G28" s="2"/>
       <c r="H28" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>87</v>
       </c>
@@ -1503,12 +1514,11 @@
         <v>12</v>
       </c>
       <c r="F29" s="1"/>
-      <c r="G29" s="2"/>
       <c r="H29" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>88</v>
       </c>
@@ -1519,12 +1529,11 @@
         <v>12</v>
       </c>
       <c r="F30" s="1"/>
-      <c r="G30" s="2"/>
       <c r="H30" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>89</v>
       </c>
@@ -1535,12 +1544,11 @@
         <v>12</v>
       </c>
       <c r="F31" s="1"/>
-      <c r="G31" s="2"/>
       <c r="H31" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>90</v>
       </c>
@@ -1551,12 +1559,11 @@
         <v>12</v>
       </c>
       <c r="F32" s="1"/>
-      <c r="G32" s="2"/>
       <c r="H32" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>91</v>
       </c>
@@ -1567,12 +1574,11 @@
         <v>12</v>
       </c>
       <c r="F33" s="1"/>
-      <c r="G33" s="2"/>
       <c r="H33" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>92</v>
       </c>
@@ -1583,12 +1589,11 @@
         <v>12</v>
       </c>
       <c r="F34" s="1"/>
-      <c r="G34" s="2"/>
       <c r="H34" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>93</v>
       </c>
@@ -1599,12 +1604,11 @@
         <v>23</v>
       </c>
       <c r="F35" s="1"/>
-      <c r="G35" s="2"/>
       <c r="H35" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>95</v>
       </c>
@@ -1615,12 +1619,11 @@
         <v>23</v>
       </c>
       <c r="F36" s="1"/>
-      <c r="G36" s="2"/>
       <c r="H36" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>96</v>
       </c>
@@ -1631,12 +1634,11 @@
         <v>23</v>
       </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="2"/>
       <c r="H37" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>97</v>
       </c>
@@ -1647,12 +1649,11 @@
         <v>12</v>
       </c>
       <c r="F38" s="1"/>
-      <c r="G38" s="2"/>
       <c r="H38" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>98</v>
       </c>
@@ -1663,12 +1664,11 @@
         <v>12</v>
       </c>
       <c r="F39" s="1"/>
-      <c r="G39" s="2"/>
       <c r="H39" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>100</v>
       </c>
@@ -1679,12 +1679,11 @@
         <v>12</v>
       </c>
       <c r="F40" s="1"/>
-      <c r="G40" s="2"/>
       <c r="H40" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>101</v>
       </c>
@@ -1695,12 +1694,11 @@
         <v>12</v>
       </c>
       <c r="F41" s="1"/>
-      <c r="G41" s="2"/>
       <c r="H41" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>102</v>
       </c>
@@ -1711,12 +1709,11 @@
         <v>23</v>
       </c>
       <c r="F42" s="1"/>
-      <c r="G42" s="2"/>
       <c r="H42" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+    <row r="43" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>103</v>
       </c>
@@ -1727,12 +1724,11 @@
         <v>23</v>
       </c>
       <c r="F43" s="1"/>
-      <c r="G43" s="2"/>
       <c r="H43" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+    <row r="44" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>104</v>
       </c>
@@ -1743,12 +1739,11 @@
         <v>12</v>
       </c>
       <c r="F44" s="1"/>
-      <c r="G44" s="2"/>
       <c r="H44" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+    <row r="45" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>105</v>
       </c>
@@ -1759,12 +1754,11 @@
         <v>12</v>
       </c>
       <c r="F45" s="1"/>
-      <c r="G45" s="2"/>
       <c r="H45" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+    <row r="46" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>106</v>
       </c>
@@ -1775,12 +1769,11 @@
         <v>23</v>
       </c>
       <c r="F46" s="1"/>
-      <c r="G46" s="2"/>
       <c r="H46" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+    <row r="47" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>107</v>
       </c>
@@ -1791,12 +1784,11 @@
         <v>12</v>
       </c>
       <c r="F47" s="1"/>
-      <c r="G47" s="2"/>
       <c r="H47" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+    <row r="48" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>108</v>
       </c>
@@ -1807,12 +1799,11 @@
         <v>12</v>
       </c>
       <c r="F48" s="1"/>
-      <c r="G48" s="2"/>
       <c r="H48" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+    <row r="49" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>109</v>
       </c>
@@ -1823,12 +1814,11 @@
         <v>23</v>
       </c>
       <c r="F49" s="1"/>
-      <c r="G49" s="2"/>
       <c r="H49" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+    <row r="50" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>110</v>
       </c>
@@ -1839,12 +1829,11 @@
         <v>23</v>
       </c>
       <c r="F50" s="1"/>
-      <c r="G50" s="2"/>
       <c r="H50" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+    <row r="51" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>112</v>
       </c>
@@ -1855,12 +1844,11 @@
         <v>12</v>
       </c>
       <c r="F51" s="1"/>
-      <c r="G51" s="2"/>
       <c r="H51" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+    <row r="52" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>113</v>
       </c>
@@ -1871,12 +1859,11 @@
         <v>12</v>
       </c>
       <c r="F52" s="1"/>
-      <c r="G52" s="2"/>
       <c r="H52" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+    <row r="53" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>114</v>
       </c>
@@ -1887,12 +1874,11 @@
         <v>12</v>
       </c>
       <c r="F53" s="1"/>
-      <c r="G53" s="2"/>
       <c r="H53" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+    <row r="54" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>115</v>
       </c>
@@ -1903,12 +1889,11 @@
         <v>12</v>
       </c>
       <c r="F54" s="1"/>
-      <c r="G54" s="2"/>
       <c r="H54" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+    <row r="55" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>116</v>
       </c>
@@ -1919,12 +1904,11 @@
         <v>12</v>
       </c>
       <c r="F55" s="1"/>
-      <c r="G55" s="2"/>
       <c r="H55" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+    <row r="56" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>117</v>
       </c>
@@ -1935,12 +1919,11 @@
         <v>12</v>
       </c>
       <c r="F56" s="1"/>
-      <c r="G56" s="2"/>
       <c r="H56" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+    <row r="57" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>118</v>
       </c>
@@ -1951,12 +1934,11 @@
         <v>12</v>
       </c>
       <c r="F57" s="1"/>
-      <c r="G57" s="2"/>
       <c r="H57" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+    <row r="58" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>119</v>
       </c>
@@ -1967,12 +1949,11 @@
         <v>12</v>
       </c>
       <c r="F58" s="1"/>
-      <c r="G58" s="2"/>
       <c r="H58" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+    <row r="59" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>120</v>
       </c>
@@ -1991,12 +1972,11 @@
       <c r="F59" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G59" s="2"/>
       <c r="H59" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+    <row r="60" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>125</v>
       </c>
@@ -2015,12 +1995,11 @@
       <c r="F60" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G60" s="2"/>
       <c r="H60" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+    <row r="61" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>129</v>
       </c>
@@ -2039,12 +2018,11 @@
       <c r="F61" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G61" s="2"/>
       <c r="H61" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+    <row r="62" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>133</v>
       </c>
@@ -2055,12 +2033,11 @@
         <v>68</v>
       </c>
       <c r="F62" s="1"/>
-      <c r="G62" s="2"/>
       <c r="H62" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+    <row r="63" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>134</v>
       </c>
@@ -2071,12 +2048,11 @@
         <v>23</v>
       </c>
       <c r="F63" s="1"/>
-      <c r="G63" s="2"/>
       <c r="H63" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+    <row r="64" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>135</v>
       </c>
@@ -2087,12 +2063,11 @@
         <v>12</v>
       </c>
       <c r="F64" s="1"/>
-      <c r="G64" s="2"/>
       <c r="H64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+    <row r="65" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>136</v>
       </c>
@@ -2103,12 +2078,11 @@
         <v>23</v>
       </c>
       <c r="F65" s="1"/>
-      <c r="G65" s="2"/>
       <c r="H65" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+    <row r="66" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>137</v>
       </c>
@@ -2119,12 +2093,11 @@
         <v>23</v>
       </c>
       <c r="F66" s="1"/>
-      <c r="G66" s="2"/>
       <c r="H66" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+    <row r="67" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>138</v>
       </c>
@@ -2135,12 +2108,11 @@
         <v>23</v>
       </c>
       <c r="F67" s="1"/>
-      <c r="G67" s="2"/>
       <c r="H67" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+    <row r="68" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>139</v>
       </c>
@@ -2151,12 +2123,11 @@
         <v>68</v>
       </c>
       <c r="F68" s="1"/>
-      <c r="G68" s="2"/>
       <c r="H68" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+    <row r="69" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>140</v>
       </c>
@@ -2167,12 +2138,11 @@
         <v>12</v>
       </c>
       <c r="F69" s="1"/>
-      <c r="G69" s="2"/>
       <c r="H69" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+    <row r="70" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>141</v>
       </c>
@@ -2183,12 +2153,11 @@
         <v>23</v>
       </c>
       <c r="F70" s="1"/>
-      <c r="G70" s="2"/>
       <c r="H70" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+    <row r="71" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>142</v>
       </c>
@@ -2199,12 +2168,11 @@
         <v>23</v>
       </c>
       <c r="F71" s="1"/>
-      <c r="G71" s="2"/>
       <c r="H71" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+    <row r="72" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>143</v>
       </c>
@@ -2215,12 +2183,11 @@
         <v>12</v>
       </c>
       <c r="F72" s="1"/>
-      <c r="G72" s="2"/>
       <c r="H72" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+    <row r="73" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>144</v>
       </c>
@@ -2231,12 +2198,11 @@
         <v>23</v>
       </c>
       <c r="F73" s="1"/>
-      <c r="G73" s="2"/>
       <c r="H73" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+    <row r="74" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>145</v>
       </c>
@@ -2247,12 +2213,11 @@
         <v>12</v>
       </c>
       <c r="F74" s="1"/>
-      <c r="G74" s="2"/>
       <c r="H74" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+    <row r="75" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>146</v>
       </c>
@@ -2263,92 +2228,66 @@
         <v>23</v>
       </c>
       <c r="F75" s="1"/>
-      <c r="G75" s="2"/>
       <c r="H75" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+    <row r="76" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
       <c r="E76" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
       <c r="H76" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="2" t="s">
+    <row r="77" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>149</v>
       </c>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
       <c r="E77" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
       <c r="H77" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
-      <c r="A78" s="2" t="s">
+    <row r="78" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>150</v>
       </c>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
       <c r="E78" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
       <c r="H78" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
-      <c r="A79" s="2" t="s">
+    <row r="79" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>151</v>
       </c>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
       <c r="E79" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
       <c r="H79" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
-      <c r="A80" s="2" t="s">
+    <row r="80" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>152</v>
       </c>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
       <c r="E80" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F80" s="2"/>
-      <c r="G80" s="2"/>
       <c r="H80" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+    <row r="81" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>153</v>
       </c>
@@ -2367,12 +2306,11 @@
       <c r="F81" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G81" s="2"/>
       <c r="H81" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+    <row r="82" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>158</v>
       </c>
@@ -2391,12 +2329,11 @@
       <c r="F82" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G82" s="2"/>
       <c r="H82" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+    <row r="83" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>162</v>
       </c>
@@ -2415,102 +2352,156 @@
       <c r="F83" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G83" s="2"/>
       <c r="H83" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+    <row r="84" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
+      <c r="E84" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H84" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+    <row r="85" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
       <c r="E85" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F85" s="2"/>
-      <c r="G85" s="2"/>
       <c r="H85" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+    <row r="86" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
       <c r="E86" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F86" s="2"/>
-      <c r="G86" s="2"/>
       <c r="H86" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+    <row r="87" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
+      <c r="E87" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H87" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+    <row r="88" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
+      <c r="E88" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H88" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="1"/>
-      <c r="F89" s="2"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="2"/>
+    <row r="89" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A89" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B89" t="s">
+        <v>173</v>
+      </c>
+      <c r="C89" t="s">
+        <v>179</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A90" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B90" t="s">
+        <v>174</v>
+      </c>
+      <c r="C90" t="s">
+        <v>180</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A91" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B91" t="s">
+        <v>177</v>
+      </c>
+      <c r="C91" t="s">
+        <v>181</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H91" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A92" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B92" t="s">
+        <v>178</v>
+      </c>
+      <c r="C92" t="s">
+        <v>182</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A93" s="5"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A94" s="5"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A95" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add new variables for health and economy
</commit_message>
<xml_diff>
--- a/backend/variables/variables.xlsx
+++ b/backend/variables/variables.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\app\ui-map-app\backend\variables\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310FA13B-1C99-4029-A811-098FD63569D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="1950" yWindow="720" windowWidth="21210" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="183">
   <si>
     <t>name</t>
   </si>
@@ -527,14 +533,49 @@
   </si>
   <si>
     <t>Transit Ridership</t>
+  </si>
+  <si>
+    <t>percentnotinsureda</t>
+  </si>
+  <si>
+    <t>percentpoverty</t>
+  </si>
+  <si>
+    <t>z_percentpoverty</t>
+  </si>
+  <si>
+    <t>z_percentnotinsureda</t>
+  </si>
+  <si>
+    <t>Population Without Health Insurance</t>
+  </si>
+  <si>
+    <t>Households Burden with Mortgage Costs</t>
+  </si>
+  <si>
+    <t>Households Burden with Rent Costs</t>
+  </si>
+  <si>
+    <t>Population Below Poverty Line</t>
+  </si>
+  <si>
+    <t>percentmortgageburdenthousehold</t>
+  </si>
+  <si>
+    <t>z_percentmortgageburdenthouseho</t>
+  </si>
+  <si>
+    <t>percentrentcostburdenthousehold</t>
+  </si>
+  <si>
+    <t>z_percentrentcostburdenthouseho</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -552,6 +593,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -582,32 +629,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -618,10 +663,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -659,71 +704,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -751,7 +796,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -774,11 +819,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -787,13 +832,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -803,7 +848,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -812,7 +857,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -821,7 +866,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -829,10 +874,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -897,24 +942,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="50.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="9.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="8.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="50.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="35" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -940,7 +983,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -959,12 +1002,11 @@
       <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2"/>
       <c r="H2" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -983,12 +1025,11 @@
       <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="2"/>
       <c r="H3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -1007,12 +1048,11 @@
       <c r="F4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="2"/>
       <c r="H4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -1023,28 +1063,22 @@
         <v>23</v>
       </c>
       <c r="F5" s="1"/>
-      <c r="G5" s="2"/>
       <c r="H5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
       <c r="E6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
       <c r="H6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1063,12 +1097,11 @@
       <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="2"/>
       <c r="H7" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -1087,12 +1120,11 @@
       <c r="F8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="2"/>
       <c r="H8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>34</v>
       </c>
@@ -1111,12 +1143,11 @@
       <c r="F9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="2"/>
       <c r="H9" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
@@ -1135,12 +1166,11 @@
       <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="2"/>
       <c r="H10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1159,12 +1189,11 @@
       <c r="F11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="2"/>
       <c r="H11" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
@@ -1183,12 +1212,11 @@
       <c r="F12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="2"/>
       <c r="H12" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -1199,28 +1227,22 @@
         <v>12</v>
       </c>
       <c r="F13" s="1"/>
-      <c r="G13" s="2"/>
       <c r="H13" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H14" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
@@ -1231,12 +1253,11 @@
         <v>23</v>
       </c>
       <c r="F15" s="1"/>
-      <c r="G15" s="2"/>
       <c r="H15" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -1247,12 +1268,11 @@
         <v>23</v>
       </c>
       <c r="F16" s="1"/>
-      <c r="G16" s="2"/>
       <c r="H16" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>55</v>
       </c>
@@ -1271,12 +1291,11 @@
       <c r="F17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="2"/>
       <c r="H17" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>59</v>
       </c>
@@ -1295,12 +1314,11 @@
       <c r="F18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="2"/>
       <c r="H18" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>63</v>
       </c>
@@ -1311,12 +1329,11 @@
         <v>12</v>
       </c>
       <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
       <c r="H19" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>64</v>
       </c>
@@ -1335,12 +1352,11 @@
       <c r="F20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="2"/>
       <c r="H20" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>69</v>
       </c>
@@ -1351,12 +1367,11 @@
         <v>23</v>
       </c>
       <c r="F21" s="1"/>
-      <c r="G21" s="2"/>
       <c r="H21" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>70</v>
       </c>
@@ -1367,12 +1382,11 @@
         <v>12</v>
       </c>
       <c r="F22" s="1"/>
-      <c r="G22" s="2"/>
       <c r="H22" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>71</v>
       </c>
@@ -1391,12 +1405,11 @@
       <c r="F23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="2"/>
       <c r="H23" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>76</v>
       </c>
@@ -1415,12 +1428,11 @@
       <c r="F24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="2"/>
       <c r="H24" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>80</v>
       </c>
@@ -1439,12 +1451,11 @@
       <c r="F25" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="2"/>
       <c r="H25" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>84</v>
       </c>
@@ -1455,12 +1466,11 @@
         <v>12</v>
       </c>
       <c r="F26" s="1"/>
-      <c r="G26" s="2"/>
       <c r="H26" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>85</v>
       </c>
@@ -1471,12 +1481,11 @@
         <v>12</v>
       </c>
       <c r="F27" s="1"/>
-      <c r="G27" s="2"/>
       <c r="H27" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>86</v>
       </c>
@@ -1487,12 +1496,11 @@
         <v>12</v>
       </c>
       <c r="F28" s="1"/>
-      <c r="G28" s="2"/>
       <c r="H28" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>87</v>
       </c>
@@ -1503,12 +1511,11 @@
         <v>12</v>
       </c>
       <c r="F29" s="1"/>
-      <c r="G29" s="2"/>
       <c r="H29" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>88</v>
       </c>
@@ -1519,12 +1526,11 @@
         <v>12</v>
       </c>
       <c r="F30" s="1"/>
-      <c r="G30" s="2"/>
       <c r="H30" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>89</v>
       </c>
@@ -1535,12 +1541,11 @@
         <v>12</v>
       </c>
       <c r="F31" s="1"/>
-      <c r="G31" s="2"/>
       <c r="H31" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>90</v>
       </c>
@@ -1551,12 +1556,11 @@
         <v>12</v>
       </c>
       <c r="F32" s="1"/>
-      <c r="G32" s="2"/>
       <c r="H32" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>91</v>
       </c>
@@ -1567,12 +1571,11 @@
         <v>12</v>
       </c>
       <c r="F33" s="1"/>
-      <c r="G33" s="2"/>
       <c r="H33" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>92</v>
       </c>
@@ -1583,12 +1586,11 @@
         <v>12</v>
       </c>
       <c r="F34" s="1"/>
-      <c r="G34" s="2"/>
       <c r="H34" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>93</v>
       </c>
@@ -1599,12 +1601,11 @@
         <v>23</v>
       </c>
       <c r="F35" s="1"/>
-      <c r="G35" s="2"/>
       <c r="H35" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>95</v>
       </c>
@@ -1615,12 +1616,11 @@
         <v>23</v>
       </c>
       <c r="F36" s="1"/>
-      <c r="G36" s="2"/>
       <c r="H36" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>96</v>
       </c>
@@ -1631,12 +1631,11 @@
         <v>23</v>
       </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="2"/>
       <c r="H37" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>97</v>
       </c>
@@ -1647,12 +1646,11 @@
         <v>12</v>
       </c>
       <c r="F38" s="1"/>
-      <c r="G38" s="2"/>
       <c r="H38" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>98</v>
       </c>
@@ -1663,12 +1661,11 @@
         <v>12</v>
       </c>
       <c r="F39" s="1"/>
-      <c r="G39" s="2"/>
       <c r="H39" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>100</v>
       </c>
@@ -1679,12 +1676,11 @@
         <v>12</v>
       </c>
       <c r="F40" s="1"/>
-      <c r="G40" s="2"/>
       <c r="H40" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>101</v>
       </c>
@@ -1695,12 +1691,11 @@
         <v>12</v>
       </c>
       <c r="F41" s="1"/>
-      <c r="G41" s="2"/>
       <c r="H41" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>102</v>
       </c>
@@ -1711,12 +1706,11 @@
         <v>23</v>
       </c>
       <c r="F42" s="1"/>
-      <c r="G42" s="2"/>
       <c r="H42" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+    <row r="43" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>103</v>
       </c>
@@ -1727,12 +1721,11 @@
         <v>23</v>
       </c>
       <c r="F43" s="1"/>
-      <c r="G43" s="2"/>
       <c r="H43" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+    <row r="44" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>104</v>
       </c>
@@ -1743,12 +1736,11 @@
         <v>12</v>
       </c>
       <c r="F44" s="1"/>
-      <c r="G44" s="2"/>
       <c r="H44" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+    <row r="45" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>105</v>
       </c>
@@ -1759,12 +1751,11 @@
         <v>12</v>
       </c>
       <c r="F45" s="1"/>
-      <c r="G45" s="2"/>
       <c r="H45" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+    <row r="46" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>106</v>
       </c>
@@ -1775,12 +1766,11 @@
         <v>23</v>
       </c>
       <c r="F46" s="1"/>
-      <c r="G46" s="2"/>
       <c r="H46" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+    <row r="47" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>107</v>
       </c>
@@ -1791,12 +1781,11 @@
         <v>12</v>
       </c>
       <c r="F47" s="1"/>
-      <c r="G47" s="2"/>
       <c r="H47" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+    <row r="48" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>108</v>
       </c>
@@ -1807,12 +1796,11 @@
         <v>12</v>
       </c>
       <c r="F48" s="1"/>
-      <c r="G48" s="2"/>
       <c r="H48" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+    <row r="49" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>109</v>
       </c>
@@ -1823,12 +1811,11 @@
         <v>23</v>
       </c>
       <c r="F49" s="1"/>
-      <c r="G49" s="2"/>
       <c r="H49" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+    <row r="50" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>110</v>
       </c>
@@ -1839,12 +1826,11 @@
         <v>23</v>
       </c>
       <c r="F50" s="1"/>
-      <c r="G50" s="2"/>
       <c r="H50" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+    <row r="51" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>112</v>
       </c>
@@ -1855,12 +1841,11 @@
         <v>12</v>
       </c>
       <c r="F51" s="1"/>
-      <c r="G51" s="2"/>
       <c r="H51" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+    <row r="52" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>113</v>
       </c>
@@ -1871,12 +1856,11 @@
         <v>12</v>
       </c>
       <c r="F52" s="1"/>
-      <c r="G52" s="2"/>
       <c r="H52" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+    <row r="53" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>114</v>
       </c>
@@ -1887,12 +1871,11 @@
         <v>12</v>
       </c>
       <c r="F53" s="1"/>
-      <c r="G53" s="2"/>
       <c r="H53" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+    <row r="54" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>115</v>
       </c>
@@ -1903,12 +1886,11 @@
         <v>12</v>
       </c>
       <c r="F54" s="1"/>
-      <c r="G54" s="2"/>
       <c r="H54" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+    <row r="55" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>116</v>
       </c>
@@ -1919,12 +1901,11 @@
         <v>12</v>
       </c>
       <c r="F55" s="1"/>
-      <c r="G55" s="2"/>
       <c r="H55" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+    <row r="56" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>117</v>
       </c>
@@ -1935,12 +1916,11 @@
         <v>12</v>
       </c>
       <c r="F56" s="1"/>
-      <c r="G56" s="2"/>
       <c r="H56" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+    <row r="57" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>118</v>
       </c>
@@ -1951,12 +1931,11 @@
         <v>12</v>
       </c>
       <c r="F57" s="1"/>
-      <c r="G57" s="2"/>
       <c r="H57" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+    <row r="58" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>119</v>
       </c>
@@ -1967,12 +1946,11 @@
         <v>12</v>
       </c>
       <c r="F58" s="1"/>
-      <c r="G58" s="2"/>
       <c r="H58" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+    <row r="59" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>120</v>
       </c>
@@ -1991,12 +1969,11 @@
       <c r="F59" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G59" s="2"/>
       <c r="H59" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+    <row r="60" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>125</v>
       </c>
@@ -2015,12 +1992,11 @@
       <c r="F60" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G60" s="2"/>
       <c r="H60" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+    <row r="61" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>129</v>
       </c>
@@ -2039,12 +2015,11 @@
       <c r="F61" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G61" s="2"/>
       <c r="H61" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+    <row r="62" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>133</v>
       </c>
@@ -2055,12 +2030,11 @@
         <v>68</v>
       </c>
       <c r="F62" s="1"/>
-      <c r="G62" s="2"/>
       <c r="H62" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+    <row r="63" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>134</v>
       </c>
@@ -2071,12 +2045,11 @@
         <v>23</v>
       </c>
       <c r="F63" s="1"/>
-      <c r="G63" s="2"/>
       <c r="H63" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+    <row r="64" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>135</v>
       </c>
@@ -2087,12 +2060,11 @@
         <v>12</v>
       </c>
       <c r="F64" s="1"/>
-      <c r="G64" s="2"/>
       <c r="H64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+    <row r="65" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>136</v>
       </c>
@@ -2103,12 +2075,11 @@
         <v>23</v>
       </c>
       <c r="F65" s="1"/>
-      <c r="G65" s="2"/>
       <c r="H65" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+    <row r="66" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>137</v>
       </c>
@@ -2119,12 +2090,11 @@
         <v>23</v>
       </c>
       <c r="F66" s="1"/>
-      <c r="G66" s="2"/>
       <c r="H66" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+    <row r="67" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>138</v>
       </c>
@@ -2135,12 +2105,11 @@
         <v>23</v>
       </c>
       <c r="F67" s="1"/>
-      <c r="G67" s="2"/>
       <c r="H67" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+    <row r="68" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>139</v>
       </c>
@@ -2151,12 +2120,11 @@
         <v>68</v>
       </c>
       <c r="F68" s="1"/>
-      <c r="G68" s="2"/>
       <c r="H68" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+    <row r="69" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>140</v>
       </c>
@@ -2167,12 +2135,11 @@
         <v>12</v>
       </c>
       <c r="F69" s="1"/>
-      <c r="G69" s="2"/>
       <c r="H69" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+    <row r="70" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>141</v>
       </c>
@@ -2183,12 +2150,11 @@
         <v>23</v>
       </c>
       <c r="F70" s="1"/>
-      <c r="G70" s="2"/>
       <c r="H70" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+    <row r="71" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>142</v>
       </c>
@@ -2199,12 +2165,11 @@
         <v>23</v>
       </c>
       <c r="F71" s="1"/>
-      <c r="G71" s="2"/>
       <c r="H71" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+    <row r="72" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>143</v>
       </c>
@@ -2215,12 +2180,11 @@
         <v>12</v>
       </c>
       <c r="F72" s="1"/>
-      <c r="G72" s="2"/>
       <c r="H72" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+    <row r="73" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>144</v>
       </c>
@@ -2231,12 +2195,11 @@
         <v>23</v>
       </c>
       <c r="F73" s="1"/>
-      <c r="G73" s="2"/>
       <c r="H73" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+    <row r="74" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>145</v>
       </c>
@@ -2247,12 +2210,11 @@
         <v>12</v>
       </c>
       <c r="F74" s="1"/>
-      <c r="G74" s="2"/>
       <c r="H74" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+    <row r="75" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>146</v>
       </c>
@@ -2263,92 +2225,66 @@
         <v>23</v>
       </c>
       <c r="F75" s="1"/>
-      <c r="G75" s="2"/>
       <c r="H75" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+    <row r="76" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
       <c r="E76" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
       <c r="H76" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="2" t="s">
+    <row r="77" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>149</v>
       </c>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
       <c r="E77" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
       <c r="H77" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
-      <c r="A78" s="2" t="s">
+    <row r="78" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>150</v>
       </c>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
       <c r="E78" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
       <c r="H78" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
-      <c r="A79" s="2" t="s">
+    <row r="79" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>151</v>
       </c>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
       <c r="E79" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
       <c r="H79" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
-      <c r="A80" s="2" t="s">
+    <row r="80" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>152</v>
       </c>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
       <c r="E80" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F80" s="2"/>
-      <c r="G80" s="2"/>
       <c r="H80" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+    <row r="81" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>153</v>
       </c>
@@ -2367,12 +2303,11 @@
       <c r="F81" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G81" s="2"/>
       <c r="H81" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+    <row r="82" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>158</v>
       </c>
@@ -2391,12 +2326,11 @@
       <c r="F82" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G82" s="2"/>
       <c r="H82" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+    <row r="83" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>162</v>
       </c>
@@ -2415,102 +2349,156 @@
       <c r="F83" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G83" s="2"/>
       <c r="H83" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+    <row r="84" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
+      <c r="E84" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H84" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+    <row r="85" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
       <c r="E85" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F85" s="2"/>
-      <c r="G85" s="2"/>
       <c r="H85" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+    <row r="86" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
       <c r="E86" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F86" s="2"/>
-      <c r="G86" s="2"/>
       <c r="H86" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+    <row r="87" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
+      <c r="E87" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H87" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+    <row r="88" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
+      <c r="E88" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H88" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="1"/>
-      <c r="F89" s="2"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="2"/>
+    <row r="89" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B89" t="s">
+        <v>171</v>
+      </c>
+      <c r="C89" t="s">
+        <v>174</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B90" t="s">
+        <v>179</v>
+      </c>
+      <c r="C90" t="s">
+        <v>180</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B91" t="s">
+        <v>181</v>
+      </c>
+      <c r="C91" t="s">
+        <v>182</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H91" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B92" t="s">
+        <v>172</v>
+      </c>
+      <c r="C92" t="s">
+        <v>173</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="4"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="4"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>